<commit_message>
fix: align one-day delivery to supplied LP and timebox guided exercises
</commit_message>
<xml_diff>
--- a/courseware/Labs/Lab-01-SPC/Starter.xlsx
+++ b/courseware/Labs/Lab-01-SPC/Starter.xlsx
@@ -717,7 +717,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Create an Excel line chart of delivery_L_h by timestamp for baseline, monitoring and pilot, with the fixed baseline mean/UCL/LCL. Flag points outside the limits without refitting them. Report phase counts and affected IDs. Explain the monitoring shift as a signal requiring investigation, not a proven restriction diagnosis. Keep invalid and missing tests visible in QualityAudit.</t>
+          <t>Review the existing Analysis and SPC_Summary chart. Keep the prepared formulas and fixed baseline limits unchanged. Identify valid monitoring points outside the limits and check one example against the source row. Return only three sentences: observed signal, supporting evidence, and an unresolved limitation. Do not rebuild the chart or calculate capability.</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Add an Excel formula RPN=S*O*D for every row. Sort a view by RPN descending while preserving mode IDs and source rows. Add a separate high-severity review flag for S&gt;=9. Create an RPN column chart. Do not treat rank or low RPN as evidence of safety acceptance.</t>
+          <t>Review the prepared FMEA_Review. Check the RPN formulas for FM01 and FM04, preserving mode IDs and provisional scores. Explain why the severity-9 row still needs review. Return one evidence gap and one proposed action for FM01; keep residual ratings unassessed. Do not rebuild the table or chart.</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Use WeeklyEvents, DefectCounts and Evidence. Draft a DMAIC table in Excel: phase, claim, metric, source, limitation, next action. Define the CTQ as delivery-test acceptance deviation, not chemical compliance. Calculate baseline and pilot rates using summed deviations divided by summed opportunities, not a simple average when denominators differ.</t>
+          <t>Review the prepared Rate_Comparison, WeeklyEvents and DMAIC tables. Check baseline and pilot rates using summed deviations divided by summed opportunities. Return three cells: measured change, limitation and next evidence. Do not create a full report or a new chart, and do not claim a causal effect from the short pilot.</t>
         </is>
       </c>
     </row>

</xml_diff>